<commit_message>
site build 2026-10-21 08:05
</commit_message>
<xml_diff>
--- a/models/sovereigns/Gulf_support_and_anchors_for_EM_sovereigns_Sovereign_Model.xlsx
+++ b/models/sovereigns/Gulf_support_and_anchors_for_EM_sovereigns_Sovereign_Model.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>as of 09-Oct-26</t>
+          <t>as of 21-Oct-26</t>
         </is>
       </c>
     </row>
@@ -590,7 +590,7 @@
       <c r="D1" t="inlineStr"/>
       <c r="E1" t="inlineStr">
         <is>
-          <t>built 19-Oct-26 by pipeline/sovereign_model.py from database/sovereigns/gulf-support-and-anchors-for-em-s.json</t>
+          <t>built 21-Oct-26 by pipeline/sovereign_model.py from database/sovereigns/gulf-support-and-anchors-for-em-s.json</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
site build 2026-10-29 08:04
</commit_message>
<xml_diff>
--- a/models/sovereigns/Gulf_support_and_anchors_for_EM_sovereigns_Sovereign_Model.xlsx
+++ b/models/sovereigns/Gulf_support_and_anchors_for_EM_sovereigns_Sovereign_Model.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>as of 21-Oct-26</t>
+          <t>as of 29-Oct-26</t>
         </is>
       </c>
     </row>
@@ -590,7 +590,7 @@
       <c r="D1" t="inlineStr"/>
       <c r="E1" t="inlineStr">
         <is>
-          <t>built 26-Oct-26 by pipeline/sovereign_model.py from database/sovereigns/gulf-support-and-anchors-for-em-s.json</t>
+          <t>built 29-Oct-26 by pipeline/sovereign_model.py from database/sovereigns/gulf-support-and-anchors-for-em-s.json</t>
         </is>
       </c>
     </row>

</xml_diff>